<commit_message>
v1.1-v1.4: QA fixes, gatepass, rate cards, bill scan, customer alerts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01788KqBCE9x4BgukbaCtAti
</commit_message>
<xml_diff>
--- a/sample_data/Intrect_invoice_export_sample.xlsx
+++ b/sample_data/Intrect_invoice_export_sample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,6 +471,26 @@
           <t>boxes</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>item_code</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>item_name</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>qty</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>line_value</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -485,7 +505,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -518,22 +538,38 @@
       </c>
       <c r="J2" t="n">
         <v>6</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>OWN-MVT</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Multivitamin Syrup 200 ml</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>24</v>
+      </c>
+      <c r="N2" t="n">
+        <v>2379.33</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>INTR-INV26-60015</t>
+          <t>INTR-INV26-60014</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>INV26-60015</t>
+          <t>INV26-60014</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -548,72 +584,296 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>P-0027</t>
+          <t>P-0044</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Sunrise Agencies</t>
+          <t>City Care Chemists</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Korba</t>
+          <t>Raipur</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>19805</v>
+        <v>7138</v>
       </c>
       <c r="J3" t="n">
-        <v>17</v>
+        <v>6</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>OWN-CET10</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Cetirizine 10 mg Tab 10s</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>396</v>
+      </c>
+      <c r="N3" t="n">
+        <v>4758.67</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>INTR-INV26-60015</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>INV26-60015</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>OWN-DIST</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>RAIPUR-HO</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>P-0027</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Sunrise Agencies</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Korba</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>19805</v>
+      </c>
+      <c r="J4" t="n">
+        <v>17</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>OWN-AZI500</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Azithromycin 500 mg Tab 3s</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>159</v>
+      </c>
+      <c r="N4" t="n">
+        <v>9902.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>INTR-INV26-60015</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>INV26-60015</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>OWN-DIST</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>RAIPUR-HO</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>P-0027</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Sunrise Agencies</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Korba</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>19805</v>
+      </c>
+      <c r="J5" t="n">
+        <v>17</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>OWN-MVT</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Multivitamin Syrup 200 ml</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>103</v>
+      </c>
+      <c r="N5" t="n">
+        <v>9902.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>INTR-INV26-60016</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>INV26-60016</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>OWN-DIST</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>RAIPUR-HO</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>P-0052</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Vardaan Pharma</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Bilaspur</t>
         </is>
       </c>
-      <c r="I4" t="n">
+      <c r="I6" t="n">
         <v>10622</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J6" t="n">
         <v>9</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>OWN-PCM650</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Paracetamol 650 mg Tab 15s</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>382</v>
+      </c>
+      <c r="N6" t="n">
+        <v>7081.33</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>INTR-INV26-60016</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>INV26-60016</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>OWN-DIST</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>RAIPUR-HO</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>P-0052</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Vardaan Pharma</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Bilaspur</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>10622</v>
+      </c>
+      <c r="J7" t="n">
+        <v>9</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>OWN-DCL</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Diclofenac Gel 30 g</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>55</v>
+      </c>
+      <c r="N7" t="n">
+        <v>3540.67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
WIP: uncommitted changes, moved to the cloud
Snapshot of the working tree the Claude desktop app took to continue
this session in the cloud. It was never committed on the desktop; fold
it into your next commit (git commit --amend) or unstage it
(git reset --mixed HEAD~1) before committing for real.
</commit_message>
<xml_diff>
--- a/sample_data/Intrect_invoice_export_sample.xlsx
+++ b/sample_data/Intrect_invoice_export_sample.xlsx
@@ -505,7 +505,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">

</xml_diff>